<commit_message>
Auto update Pengadaan 2026-10-06 08:08:44
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-06).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-06).xlsx
@@ -1020,35 +1020,27 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>1796500000</v>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1389,22 +1381,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="D25" s="11" t="n">
         <v>677290237</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="F25" s="11" t="n">
         <v>137583844</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>116218702</v>
+        <v>1301651478</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>90</v>
@@ -1528,13 +1520,13 @@
         <v>170</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2230970155</v>
+        <v>2221466002</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1136240668</v>
+        <v>1126736515</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1868,13 +1860,13 @@
         <v>112</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1305525621</v>
+        <v>1279995621</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>18</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>378058156</v>
+        <v>352528156</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>18</v>
@@ -2035,22 +2027,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>141795000</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>64745634</v>
+        <v>121094174</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>17</v>
@@ -3363,22 +3355,22 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3937</v>
+        <v>3964</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32744774956</v>
+        <v>32709740803</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>417</v>
+        <v>444</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6693854006</v>
+        <v>6658819853</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>417</v>
+        <v>444</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>6159636368.6</v>
+        <v>9197917684.6</v>
       </c>
       <c r="I77" s="12" t="n">
         <v>3520</v>
@@ -5584,28 +5576,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>595373450</v>
+        <v>379426400</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>417917650</v>
+        <v>201970600</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>198768000</v>
+        <v>142419460</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>198768000</v>
+        <v>142419460</v>
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
@@ -7536,28 +7528,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>97487528498</v>
+        <v>97271581448</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>64871532693</v>
+        <v>64655585643</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>63154109969.41</v>
+        <v>63097761429.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>33555205925</v>
+        <v>33498857385</v>
       </c>
       <c r="K77" s="12" t="n">
         <v>12</v>
@@ -8371,28 +8363,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>26035273641</v>
+        <v>24238773641</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>26035273641</v>
+        <v>24238773641</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8590,13 +8582,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8815,34 +8807,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>48003814160</v>
+        <v>5652342335</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>47632716881</v>
+        <v>5281245056</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>4157004750</v>
+        <v>2971571974</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>4157004750</v>
+        <v>2971571974</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>2945468782</v>
+        <v>1854621974</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -12013,34 +12005,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>238</v>
+        <v>214</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>179940571818</v>
+        <v>135505209081</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>158</v>
+        <v>134</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>143234386443</v>
+        <v>98799023706</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>158</v>
+        <v>134</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>69752277713.01001</v>
+        <v>66770344937.01</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>139</v>
+        <v>115</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>65303843913</v>
+        <v>62321911137</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>4005987066</v>
+        <v>2915140258</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>80</v>

</xml_diff>

<commit_message>
Auto update Pengadaan 2026-10-06 10:10:09
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-06).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-06).xlsx
@@ -1020,27 +1020,35 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
-        <v>1</v>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
-        <v>1</v>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>1796500000</v>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1381,22 +1389,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>126</v>
+        <v>103</v>
       </c>
       <c r="D25" s="11" t="n">
         <v>677290237</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="F25" s="11" t="n">
         <v>137583844</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>1301651478</v>
+        <v>116218702</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>90</v>
@@ -1520,13 +1528,13 @@
         <v>170</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2221466002</v>
+        <v>2230970155</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1126736515</v>
+        <v>1136240668</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1860,13 +1868,13 @@
         <v>112</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1279995621</v>
+        <v>1305525621</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>18</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>352528156</v>
+        <v>378058156</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>18</v>
@@ -2027,22 +2035,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>141795000</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>121094174</v>
+        <v>64745634</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>17</v>
@@ -3355,22 +3363,22 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3964</v>
+        <v>3937</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32709740803</v>
+        <v>32744774956</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>444</v>
+        <v>417</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6658819853</v>
+        <v>6693854006</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>444</v>
+        <v>417</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>9197917684.6</v>
+        <v>6159636368.6</v>
       </c>
       <c r="I77" s="12" t="n">
         <v>3520</v>
@@ -5576,28 +5584,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D44" s="9" t="n">
+        <v>595373450</v>
+      </c>
+      <c r="E44" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="D44" s="9" t="n">
-        <v>379426400</v>
-      </c>
-      <c r="E44" s="7" t="n">
-        <v>2</v>
-      </c>
       <c r="F44" s="9" t="n">
-        <v>201970600</v>
+        <v>417917650</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>142419460</v>
+        <v>198768000</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>142419460</v>
+        <v>198768000</v>
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
@@ -7528,28 +7536,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>821</v>
+        <v>824</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>97271581448</v>
+        <v>97487528498</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>64655585643</v>
+        <v>64871532693</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>63097761429.41</v>
+        <v>63154109969.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>33498857385</v>
+        <v>33555205925</v>
       </c>
       <c r="K77" s="12" t="n">
         <v>12</v>
@@ -8363,28 +8371,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>25286544212</v>
+        <v>26735477939</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>25286544212</v>
+        <v>26735477939</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>24238773641</v>
+        <v>26035273641</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>24238773641</v>
+        <v>26035273641</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8582,13 +8590,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8807,34 +8815,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>5652342335</v>
+        <v>48003814160</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>5281245056</v>
+        <v>47632716881</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>1854621974</v>
+        <v>2945468782</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -12005,34 +12013,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>214</v>
+        <v>238</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>135505209081</v>
+        <v>179940571818</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>98799023706</v>
+        <v>143234386443</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>66770344937.01</v>
+        <v>69752277713.01001</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>62321911137</v>
+        <v>65303843913</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>2915140258</v>
+        <v>4005987066</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>80</v>

</xml_diff>

<commit_message>
Auto update Pengadaan 2026-10-06 12:10:29
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-06).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-06).xlsx
@@ -1020,35 +1020,27 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>1796500000</v>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1389,22 +1381,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="D25" s="11" t="n">
         <v>677290237</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="F25" s="11" t="n">
         <v>137583844</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>116218702</v>
+        <v>1301651478</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>90</v>
@@ -1528,13 +1520,13 @@
         <v>170</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2230970155</v>
+        <v>2221466002</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1136240668</v>
+        <v>1126736515</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1868,13 +1860,13 @@
         <v>112</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1305525621</v>
+        <v>1279995621</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>18</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>378058156</v>
+        <v>352528156</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>18</v>
@@ -2035,22 +2027,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>141795000</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>64745634</v>
+        <v>121094174</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>17</v>
@@ -3363,22 +3355,22 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3937</v>
+        <v>3964</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32744774956</v>
+        <v>32709740803</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>417</v>
+        <v>444</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6693854006</v>
+        <v>6658819853</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>417</v>
+        <v>444</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>6159636368.6</v>
+        <v>9197917684.6</v>
       </c>
       <c r="I77" s="12" t="n">
         <v>3520</v>
@@ -5584,28 +5576,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>595373450</v>
+        <v>379426400</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>417917650</v>
+        <v>201970600</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>198768000</v>
+        <v>142419460</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>198768000</v>
+        <v>142419460</v>
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
@@ -7536,28 +7528,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>97487528498</v>
+        <v>97271581448</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>64871532693</v>
+        <v>64655585643</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>63154109969.41</v>
+        <v>63097761429.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>33555205925</v>
+        <v>33498857385</v>
       </c>
       <c r="K77" s="12" t="n">
         <v>12</v>
@@ -8371,28 +8363,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>26035273641</v>
+        <v>24238773641</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>26035273641</v>
+        <v>24238773641</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8590,13 +8582,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8815,34 +8807,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>48003814160</v>
+        <v>5652342335</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>47632716881</v>
+        <v>5281245056</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>4157004750</v>
+        <v>2971571974</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>4157004750</v>
+        <v>2971571974</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>2945468782</v>
+        <v>1854621974</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -12013,34 +12005,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>238</v>
+        <v>214</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>179940571818</v>
+        <v>135505209081</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>158</v>
+        <v>134</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>143234386443</v>
+        <v>98799023706</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>158</v>
+        <v>134</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>69752277713.01001</v>
+        <v>66770344937.01</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>139</v>
+        <v>115</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>65303843913</v>
+        <v>62321911137</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>4005987066</v>
+        <v>2915140258</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>80</v>

</xml_diff>